<commit_message>
Updated Day 01 with additional formatting practice sheets
</commit_message>
<xml_diff>
--- a/Excel_Introduction_and_Data_Formating/Day_01_Introduction & Data_Formating.xlsx
+++ b/Excel_Introduction_and_Data_Formating/Day_01_Introduction & Data_Formating.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e01621777f20dcb/Desktop/Excel_For_Data_Analytics/Excel_Introduction_and_Data_Formating/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="454" documentId="8_{5BFF8888-E61D-45DF-9242-3D43603A95FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{842F9622-8709-4840-ACB5-6BE6D18335F4}"/>
+  <xr:revisionPtr revIDLastSave="737" documentId="8_{5BFF8888-E61D-45DF-9242-3D43603A95FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1299FC30-E773-41C0-9180-860B31019693}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{E6744EAD-35E1-4258-81F8-3CB7F274373C}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="3" xr2:uid="{E6744EAD-35E1-4258-81F8-3CB7F274373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Excel Interface" sheetId="1" r:id="rId1"/>
-    <sheet name="Text Formating " sheetId="2" r:id="rId2"/>
+    <sheet name="Data Formating " sheetId="2" r:id="rId2"/>
+    <sheet name="Data Type" sheetId="3" r:id="rId3"/>
+    <sheet name="sorting and Filtering" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="121">
   <si>
     <t>1.edit in data  (F2)/double click</t>
   </si>
@@ -181,9 +183,6 @@
     <t>Display worksheet information</t>
   </si>
   <si>
-    <t>Data set</t>
-  </si>
-  <si>
     <t>Department</t>
   </si>
   <si>
@@ -241,9 +240,6 @@
     <t>Banglore</t>
   </si>
   <si>
-    <t>Number Formatting</t>
-  </si>
-  <si>
     <t xml:space="preserve">Product </t>
   </si>
   <si>
@@ -335,13 +331,87 @@
   </si>
   <si>
     <t>used to enter/edit formulas</t>
+  </si>
+  <si>
+    <t>Text Data Type</t>
+  </si>
+  <si>
+    <t>Data Formating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numeric data type </t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Dec</t>
+  </si>
+  <si>
+    <t>step  of data type: home -&gt;Number&gt;-Genral</t>
+  </si>
+  <si>
+    <t>sanya</t>
+  </si>
+  <si>
+    <t>keshav</t>
+  </si>
+  <si>
+    <t>rajan</t>
+  </si>
+  <si>
+    <t>satyam</t>
+  </si>
+  <si>
+    <t>kittu</t>
+  </si>
+  <si>
+    <t>LOW TO HIGH</t>
+  </si>
+  <si>
+    <t>HIGH TO LOW</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="169" formatCode="&quot;₹&quot;\ #,##0"/>
+    <numFmt numFmtId="170" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+  </numFmts>
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,6 +450,27 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -407,8 +498,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -441,13 +556,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7030A0"/>
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -471,12 +592,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -493,8 +608,62 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -517,11 +686,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color theme="1"/>
+      </left>
+      <right style="thick">
+        <color theme="1"/>
+      </right>
+      <top style="thick">
+        <color theme="1"/>
+      </top>
+      <bottom style="thick">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -542,9 +736,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -560,62 +751,110 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="1" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="1" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -989,30 +1228,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="A1" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="A2" s="34"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
     </row>
     <row r="3" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="37"/>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
+      <c r="A3" s="34"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
       <c r="G3" s="7" t="s">
         <v>0</v>
       </c>
@@ -1049,7 +1288,7 @@
       <c r="K6" s="7"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C7" s="12"/>
+      <c r="C7" s="11"/>
       <c r="E7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1065,7 +1304,7 @@
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="28"/>
+      <c r="C8" s="25"/>
       <c r="D8" s="2">
         <v>1</v>
       </c>
@@ -1089,7 +1328,7 @@
       <c r="F9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="11" t="s">
         <v>29</v>
       </c>
       <c r="I9" s="5" t="s">
@@ -1135,7 +1374,7 @@
       <c r="I11" t="s">
         <v>42</v>
       </c>
-      <c r="J11" s="11"/>
+      <c r="J11" s="10"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D12" s="2">
@@ -1147,16 +1386,16 @@
       <c r="F12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="9"/>
+      <c r="G12" s="8"/>
       <c r="H12" t="s">
         <v>33</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
       <c r="N12" s="6"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -1169,16 +1408,16 @@
       <c r="F13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="10"/>
-      <c r="H13" s="13" t="s">
+      <c r="G13" s="9"/>
+      <c r="H13" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D14" s="2">
@@ -1190,16 +1429,16 @@
       <c r="F14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="10"/>
-      <c r="H14" s="14" t="s">
+      <c r="G14" s="9"/>
+      <c r="H14" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="I14" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D15" s="2">
@@ -1208,16 +1447,16 @@
       <c r="E15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="10"/>
-      <c r="H15" s="14" t="s">
+      <c r="G15" s="9"/>
+      <c r="H15" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="I15" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D16" s="2">
@@ -1226,16 +1465,16 @@
       <c r="E16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G16" s="10"/>
-      <c r="H16" s="15" t="s">
+      <c r="G16" s="9"/>
+      <c r="H16" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="I16" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
+      <c r="I16" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
     </row>
     <row r="17" spans="4:12" x14ac:dyDescent="0.3">
       <c r="D17" s="2">
@@ -1244,16 +1483,16 @@
       <c r="E17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="15" t="s">
+      <c r="G17" s="9"/>
+      <c r="H17" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="I17" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
+      <c r="I17" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
     </row>
     <row r="18" spans="4:12" x14ac:dyDescent="0.3">
       <c r="D18" s="2">
@@ -1262,16 +1501,16 @@
       <c r="E18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="15" t="s">
+      <c r="G18" s="9"/>
+      <c r="H18" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I18" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
+      <c r="I18" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
     </row>
     <row r="19" spans="4:12" x14ac:dyDescent="0.3">
       <c r="D19" s="2">
@@ -1280,34 +1519,34 @@
       <c r="E19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="10"/>
-      <c r="H19" s="15" t="s">
+      <c r="G19" s="9"/>
+      <c r="H19" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="I19" s="15" t="s">
+      <c r="I19" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
     </row>
     <row r="20" spans="4:12" x14ac:dyDescent="0.3">
-      <c r="G20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="G20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
     </row>
     <row r="21" spans="4:12" x14ac:dyDescent="0.3">
-      <c r="G21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
+      <c r="G21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
     </row>
     <row r="22" spans="4:12" x14ac:dyDescent="0.3">
-      <c r="G22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
+      <c r="G22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1329,12 +1568,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4BF2667-FA00-42BA-A9F8-94619B32ED44}">
-  <dimension ref="C3:L23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.21875" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" customWidth="1"/>
     <col min="10" max="10" width="7.33203125" customWidth="1"/>
@@ -1342,437 +1581,1106 @@
     <col min="12" max="12" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="D3" s="18" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="D3" s="36"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+    </row>
+    <row r="4" spans="1:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="38"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+    </row>
+    <row r="5" spans="1:18" ht="21" x14ac:dyDescent="0.35">
+      <c r="C5" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+    </row>
+    <row r="6" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+      <c r="C6" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-    </row>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="I4" s="26" t="s">
+      <c r="E6" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="42" t="s">
+        <v>75</v>
+      </c>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="39"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C7" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C8" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="J8" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-    </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-    </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C6" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C7" s="19" t="s">
+      <c r="K8" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="L8" s="26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C9" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="27">
+        <v>101</v>
+      </c>
+      <c r="I9" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="J9" s="31">
+        <v>21</v>
+      </c>
+      <c r="K9" s="32">
+        <v>20000</v>
+      </c>
+      <c r="L9" s="33" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C10" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" s="27">
+        <v>102</v>
+      </c>
+      <c r="I10" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="J10" s="31">
+        <v>22</v>
+      </c>
+      <c r="K10" s="32">
+        <v>25000</v>
+      </c>
+      <c r="L10" s="33" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C11" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" s="27">
+        <v>103</v>
+      </c>
+      <c r="I11" s="29" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11" s="31">
+        <v>21</v>
+      </c>
+      <c r="K11" s="32">
+        <v>40000</v>
+      </c>
+      <c r="L11" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="1" t="s">
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C12" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="20" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C8" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="E12" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="27">
+        <v>104</v>
+      </c>
+      <c r="I12" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="J12" s="31">
+        <v>24</v>
+      </c>
+      <c r="K12" s="32">
+        <v>45000</v>
+      </c>
+      <c r="L12" s="33" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H13" s="27">
+        <v>105</v>
+      </c>
+      <c r="I13" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="J13" s="31">
+        <v>28</v>
+      </c>
+      <c r="K13" s="32">
+        <v>30000</v>
+      </c>
+      <c r="L13" s="33" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H14" s="27">
+        <v>106</v>
+      </c>
+      <c r="I14" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="J14" s="31">
+        <v>30</v>
+      </c>
+      <c r="K14" s="32">
+        <v>95000</v>
+      </c>
+      <c r="L14" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="I8" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="J8" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="K8" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C9" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="H9" s="30">
-        <v>101</v>
-      </c>
-      <c r="I9" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="J9" s="34">
-        <v>21</v>
-      </c>
-      <c r="K9" s="35">
-        <v>20000</v>
-      </c>
-      <c r="L9" s="36" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C10" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="1" t="s">
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H15" s="27">
+        <v>107</v>
+      </c>
+      <c r="I15" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="J15" s="31">
+        <v>27</v>
+      </c>
+      <c r="K15" s="32">
+        <v>60000</v>
+      </c>
+      <c r="L15" s="33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="H16" s="27">
+        <v>108</v>
+      </c>
+      <c r="I16" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="J16" s="31">
+        <v>29</v>
+      </c>
+      <c r="K16" s="32">
+        <v>55000</v>
+      </c>
+      <c r="L16" s="33" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="3:12" ht="15" x14ac:dyDescent="0.35">
+      <c r="C17" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+      <c r="H17" s="27">
+        <v>109</v>
+      </c>
+      <c r="I17" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="J17" s="31">
+        <v>20</v>
+      </c>
+      <c r="K17" s="32">
+        <v>34000</v>
+      </c>
+      <c r="L17" s="33" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C18" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="H18" s="28">
+        <v>110</v>
+      </c>
+      <c r="I18" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="J18" s="31">
+        <v>27</v>
+      </c>
+      <c r="K18" s="32">
+        <v>23000</v>
+      </c>
+      <c r="L18" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="E10" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10" s="30">
-        <v>102</v>
-      </c>
-      <c r="I10" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="J10" s="34">
-        <v>22</v>
-      </c>
-      <c r="K10" s="35">
-        <v>25000</v>
-      </c>
-      <c r="L10" s="36" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C11" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="H11" s="30">
-        <v>103</v>
-      </c>
-      <c r="I11" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="J11" s="34">
-        <v>21</v>
-      </c>
-      <c r="K11" s="35">
-        <v>40000</v>
-      </c>
-      <c r="L11" s="36" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C12" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="H12" s="30">
-        <v>104</v>
-      </c>
-      <c r="I12" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="J12" s="34">
-        <v>24</v>
-      </c>
-      <c r="K12" s="35">
-        <v>45000</v>
-      </c>
-      <c r="L12" s="36" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="13" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="H13" s="30">
-        <v>105</v>
-      </c>
-      <c r="I13" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="J13" s="34">
-        <v>28</v>
-      </c>
-      <c r="K13" s="35">
-        <v>30000</v>
-      </c>
-      <c r="L13" s="36" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="30">
-        <v>106</v>
-      </c>
-      <c r="I14" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="J14" s="34">
-        <v>30</v>
-      </c>
-      <c r="K14" s="35">
-        <v>95000</v>
-      </c>
-      <c r="L14" s="36" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="30">
-        <v>107</v>
-      </c>
-      <c r="I15" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="J15" s="34">
-        <v>27</v>
-      </c>
-      <c r="K15" s="35">
-        <v>60000</v>
-      </c>
-      <c r="L15" s="36" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="D16" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="H16" s="30">
-        <v>108</v>
-      </c>
-      <c r="I16" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="J16" s="34">
-        <v>29</v>
-      </c>
-      <c r="K16" s="35">
-        <v>55000</v>
-      </c>
-      <c r="L16" s="36" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="H17" s="30">
-        <v>109</v>
-      </c>
-      <c r="I17" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="J17" s="34">
-        <v>20</v>
-      </c>
-      <c r="K17" s="35">
-        <v>34000</v>
-      </c>
-      <c r="L17" s="36" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C18" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="22" t="s">
+    </row>
+    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
+      <c r="C19" s="22" t="s">
         <v>71</v>
-      </c>
-      <c r="F18" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="H18" s="31">
-        <v>110</v>
-      </c>
-      <c r="I18" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="J18" s="34">
-        <v>27</v>
-      </c>
-      <c r="K18" s="35">
-        <v>23000</v>
-      </c>
-      <c r="L18" s="36" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C19" s="23" t="s">
-        <v>73</v>
       </c>
       <c r="D19" s="1">
         <v>65000</v>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="23">
         <v>0.1</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="24">
         <v>58500</v>
       </c>
-      <c r="H19" s="30">
+      <c r="H19" s="27">
         <v>111</v>
       </c>
-      <c r="I19" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="J19" s="34">
+      <c r="I19" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="J19" s="31">
         <v>26</v>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="32">
         <v>23000</v>
       </c>
-      <c r="L19" s="36" t="s">
-        <v>59</v>
+      <c r="L19" s="33" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C20" s="23" t="s">
-        <v>74</v>
+      <c r="C20" s="22" t="s">
+        <v>72</v>
       </c>
       <c r="D20" s="1">
         <v>25000</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="23">
         <v>0.05</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="24">
         <v>23750</v>
       </c>
-      <c r="H20" s="30">
+      <c r="H20" s="27">
         <v>112</v>
       </c>
-      <c r="I20" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="J20" s="34">
+      <c r="I20" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="J20" s="31">
         <v>29</v>
       </c>
-      <c r="K20" s="35">
+      <c r="K20" s="32">
         <v>34530</v>
       </c>
-      <c r="L20" s="36" t="s">
-        <v>57</v>
+      <c r="L20" s="33" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C21" s="23" t="s">
-        <v>75</v>
+      <c r="C21" s="22" t="s">
+        <v>73</v>
       </c>
       <c r="D21" s="1">
         <v>800</v>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="23">
         <v>0.08</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="24">
         <v>736</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="27">
         <v>113</v>
       </c>
-      <c r="I21" s="32" t="s">
-        <v>91</v>
-      </c>
-      <c r="J21" s="34">
+      <c r="I21" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="J21" s="31">
         <v>25</v>
       </c>
-      <c r="K21" s="35">
+      <c r="K21" s="32">
         <v>80000</v>
       </c>
-      <c r="L21" s="36" t="s">
-        <v>58</v>
+      <c r="L21" s="33" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="C22" s="23" t="s">
-        <v>76</v>
+      <c r="C22" s="22" t="s">
+        <v>74</v>
       </c>
       <c r="D22" s="1">
         <v>1500</v>
       </c>
-      <c r="E22" s="24">
+      <c r="E22" s="23">
         <v>0.12</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="24">
         <v>1320</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="27">
         <v>114</v>
       </c>
-      <c r="I22" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="J22" s="34">
+      <c r="I22" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="J22" s="31">
         <v>23</v>
       </c>
-      <c r="K22" s="35">
+      <c r="K22" s="32">
         <v>76000</v>
       </c>
-      <c r="L22" s="36" t="s">
-        <v>58</v>
+      <c r="L22" s="33" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="3:12" x14ac:dyDescent="0.3">
-      <c r="H23" s="30">
+      <c r="H23" s="27">
         <v>115</v>
       </c>
-      <c r="I23" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="J23" s="34">
+      <c r="I23" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="J23" s="31">
         <v>22</v>
       </c>
-      <c r="K23" s="35">
+      <c r="K23" s="32">
         <v>65000</v>
       </c>
-      <c r="L23" s="36" t="s">
-        <v>58</v>
+      <c r="L23" s="33" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="I4:K5"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="H6:L6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FA472E3-E66D-43B0-85D6-FCDF14D5A812}">
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+    </row>
+    <row r="2" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="45">
+        <v>2</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="F3" s="47">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="45">
+        <v>3</v>
+      </c>
+      <c r="D4" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="47">
+        <v>46205</v>
+      </c>
+      <c r="H4" s="48">
+        <v>100</v>
+      </c>
+      <c r="J4" s="49">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="45">
+        <v>4</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" s="47">
+        <v>46206</v>
+      </c>
+      <c r="H5" s="48">
+        <v>230</v>
+      </c>
+      <c r="J5" s="49">
+        <v>230</v>
+      </c>
+      <c r="L5" s="50">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="45">
+        <v>5</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="F6" s="47">
+        <v>46207</v>
+      </c>
+      <c r="H6" s="48">
+        <v>300</v>
+      </c>
+      <c r="J6" s="49">
+        <v>300</v>
+      </c>
+      <c r="L6" s="50">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="45">
+        <v>6</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" s="47">
+        <v>46208</v>
+      </c>
+      <c r="H7" s="48">
+        <v>400</v>
+      </c>
+      <c r="J7" s="49">
+        <v>400</v>
+      </c>
+      <c r="L7" s="50">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="45">
+        <v>7</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" s="47">
+        <v>46209</v>
+      </c>
+      <c r="H8" s="48">
+        <v>360</v>
+      </c>
+      <c r="J8" s="49">
+        <v>360</v>
+      </c>
+      <c r="L8" s="50">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="45">
+        <v>8</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="F9" s="47">
+        <v>46210</v>
+      </c>
+      <c r="H9" s="48">
+        <v>432</v>
+      </c>
+      <c r="J9" s="49">
+        <v>432</v>
+      </c>
+      <c r="L9" s="50">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="45">
+        <v>9</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" s="47">
+        <v>46211</v>
+      </c>
+      <c r="H10" s="48">
+        <v>150</v>
+      </c>
+      <c r="J10" s="49">
+        <v>150</v>
+      </c>
+      <c r="L10" s="50">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="45">
+        <v>10</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" s="47">
+        <v>46212</v>
+      </c>
+      <c r="H11" s="48">
+        <v>300</v>
+      </c>
+      <c r="J11" s="49">
+        <v>300</v>
+      </c>
+      <c r="L11" s="50">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="45">
+        <v>11</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="F12" s="47">
+        <v>46213</v>
+      </c>
+      <c r="H12" s="48">
+        <v>350</v>
+      </c>
+      <c r="J12" s="49">
+        <v>350</v>
+      </c>
+      <c r="L12" s="50">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="45">
+        <v>12</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>111</v>
+      </c>
+      <c r="F13" s="47">
+        <v>46214</v>
+      </c>
+      <c r="H13" s="48">
+        <v>600</v>
+      </c>
+      <c r="J13" s="49">
+        <v>600</v>
+      </c>
+      <c r="L13" s="50">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="45">
+        <v>13</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="F14" s="47">
+        <v>46215</v>
+      </c>
+      <c r="L14" s="50">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="45">
+        <v>14</v>
+      </c>
+      <c r="F15" s="47">
+        <v>46216</v>
+      </c>
+      <c r="L15" s="50">
+        <v>46214</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="45">
+        <v>15</v>
+      </c>
+      <c r="F16" s="47">
+        <v>46217</v>
+      </c>
+      <c r="L16" s="50">
+        <v>46215</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="45">
+        <v>16</v>
+      </c>
+      <c r="F17" s="47">
+        <v>46218</v>
+      </c>
+      <c r="L17" s="50">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="45">
+        <v>17</v>
+      </c>
+      <c r="F18" s="47">
+        <v>46219</v>
+      </c>
+      <c r="L18" s="50">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="45">
+        <v>18</v>
+      </c>
+      <c r="F19" s="47">
+        <v>46220</v>
+      </c>
+      <c r="L19" s="50">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="45">
+        <v>19</v>
+      </c>
+      <c r="F20" s="47">
+        <v>46221</v>
+      </c>
+      <c r="L20" s="50">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="45">
+        <v>20</v>
+      </c>
+      <c r="L21" s="50">
+        <v>46220</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="45">
+        <v>21</v>
+      </c>
+      <c r="L22" s="50">
+        <v>46221</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="45">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="45">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="45">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="45">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1964190-7CB5-401C-8B71-AC95BAD6EF8F}">
+  <dimension ref="A2:J21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:10" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C3" s="47">
+        <v>46221</v>
+      </c>
+      <c r="D3" s="58" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="47">
+        <v>46220</v>
+      </c>
+      <c r="D4" s="58"/>
+    </row>
+    <row r="5" spans="1:10" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="47">
+        <v>46219</v>
+      </c>
+      <c r="D5" s="58"/>
+      <c r="E5" s="49">
+        <v>600</v>
+      </c>
+      <c r="F5" s="57" t="s">
+        <v>120</v>
+      </c>
+      <c r="G5" s="53">
+        <v>0.1</v>
+      </c>
+      <c r="H5" s="54" t="s">
+        <v>119</v>
+      </c>
+      <c r="I5" s="56" t="s">
+        <v>114</v>
+      </c>
+      <c r="J5" s="55" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="46" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="47">
+        <v>46218</v>
+      </c>
+      <c r="D6" s="58"/>
+      <c r="E6" s="49">
+        <v>432</v>
+      </c>
+      <c r="F6" s="57"/>
+      <c r="G6" s="52">
+        <v>0.3</v>
+      </c>
+      <c r="H6" s="54"/>
+      <c r="I6" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="J6" s="55"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="47">
+        <v>46217</v>
+      </c>
+      <c r="D7" s="58"/>
+      <c r="E7" s="49">
+        <v>400</v>
+      </c>
+      <c r="F7" s="57"/>
+      <c r="G7" s="52">
+        <v>0.34</v>
+      </c>
+      <c r="H7" s="54"/>
+      <c r="I7" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="J7" s="55"/>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="47">
+        <v>46216</v>
+      </c>
+      <c r="D8" s="58"/>
+      <c r="E8" s="49">
+        <v>360</v>
+      </c>
+      <c r="F8" s="57"/>
+      <c r="G8" s="52">
+        <v>0.43</v>
+      </c>
+      <c r="H8" s="54"/>
+      <c r="I8" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="J8" s="55"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="47">
+        <v>46215</v>
+      </c>
+      <c r="D9" s="58"/>
+      <c r="E9" s="49">
+        <v>350</v>
+      </c>
+      <c r="F9" s="57"/>
+      <c r="G9" s="52">
+        <v>0.45</v>
+      </c>
+      <c r="H9" s="54"/>
+      <c r="I9" s="51" t="s">
+        <v>118</v>
+      </c>
+      <c r="J9" s="55"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="47">
+        <v>46214</v>
+      </c>
+      <c r="D10" s="58"/>
+      <c r="E10" s="49">
+        <v>300</v>
+      </c>
+      <c r="F10" s="57"/>
+      <c r="G10" s="52">
+        <v>0.5</v>
+      </c>
+      <c r="H10" s="54"/>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="47">
+        <v>46213</v>
+      </c>
+      <c r="D11" s="58"/>
+      <c r="E11" s="49">
+        <v>300</v>
+      </c>
+      <c r="F11" s="57"/>
+      <c r="G11" s="52">
+        <v>0.6</v>
+      </c>
+      <c r="H11" s="54"/>
+    </row>
+    <row r="12" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="47">
+        <v>46212</v>
+      </c>
+      <c r="D12" s="58"/>
+      <c r="E12" s="49">
+        <v>230</v>
+      </c>
+      <c r="F12" s="57"/>
+      <c r="G12" s="52">
+        <v>0.9</v>
+      </c>
+      <c r="H12" s="54"/>
+    </row>
+    <row r="13" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="47">
+        <v>46211</v>
+      </c>
+      <c r="D13" s="58"/>
+      <c r="E13" s="49">
+        <v>150</v>
+      </c>
+      <c r="F13" s="57"/>
+    </row>
+    <row r="14" spans="1:10" ht="15.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="C14" s="47">
+        <v>46210</v>
+      </c>
+      <c r="D14" s="58"/>
+      <c r="E14" s="49">
+        <v>100</v>
+      </c>
+      <c r="F14" s="57"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="46" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="47">
+        <v>46209</v>
+      </c>
+      <c r="D15" s="58"/>
+    </row>
+    <row r="16" spans="1:10" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="47">
+        <v>46208</v>
+      </c>
+      <c r="D16" s="58"/>
+    </row>
+    <row r="17" spans="3:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C17" s="47">
+        <v>46207</v>
+      </c>
+      <c r="D17" s="58"/>
+    </row>
+    <row r="18" spans="3:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C18" s="47">
+        <v>46206</v>
+      </c>
+      <c r="D18" s="58"/>
+    </row>
+    <row r="19" spans="3:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C19" s="47">
+        <v>46205</v>
+      </c>
+      <c r="D19" s="58"/>
+    </row>
+    <row r="20" spans="3:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C20" s="47">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C3:C20">
+    <sortCondition descending="1" ref="C3:C20"/>
+  </sortState>
+  <mergeCells count="4">
+    <mergeCell ref="H5:H12"/>
+    <mergeCell ref="J5:J9"/>
+    <mergeCell ref="F5:F14"/>
+    <mergeCell ref="D3:D19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>